<commit_message>
Expand image prompts to 20/section on 4 videos, add content/prompt creation-date tracking
SoftChic60 (boot-mistakes, blouse-mistakes) and Viva Estilo (relojes, panuelo)
each had far too few image prompts per section (~5-12 instead of 20). Regenerated
all four videos' image-prompts-FULL.txt (and Viva Estilo's per-section
image-prompts/ files) to a consistent 20 prompts per section. Also added
"Ngay tao content" / "Ngay tao prompt anh" columns to both channels' plan
sheets so future sessions can see when each video's script and prompts were
(re-)generated.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/channels/soft-chic-60/output/softchic60-content-plan.xlsx
+++ b/channels/soft-chic-60/output/softchic60-content-plan.xlsx
@@ -2853,7 +2853,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:R11"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2903,6 +2907,12 @@
       </c>
       <c r="P1" t="str">
         <v>Đã xuất content?</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Ngày tạo content</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Ngày tạo prompt ảnh</v>
       </c>
     </row>
     <row r="2" xml:space="preserve">
@@ -2962,6 +2972,12 @@
       <c r="P2" t="str">
         <v>✅ Đã xuất (kịch bản đầy đủ + ảnh)</v>
       </c>
+      <c r="Q2" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="R2" t="str">
+        <v>2026-09-08</v>
+      </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3">
@@ -3018,6 +3034,12 @@
       <c r="P3" t="str">
         <v>Chưa xuất</v>
       </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4">
@@ -3073,6 +3095,12 @@
       </c>
       <c r="P4" t="str">
         <v>Chưa xuất</v>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -3131,6 +3159,12 @@
       </c>
       <c r="P5" t="str">
         <v>Chưa xuất</v>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -3191,6 +3225,12 @@
       <c r="P6" t="str">
         <v>Chưa xuất</v>
       </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7">
@@ -3248,6 +3288,12 @@
       <c r="P7" t="str">
         <v>Chưa xuất</v>
       </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8" xml:space="preserve">
       <c r="A8">
@@ -3303,6 +3349,12 @@
       </c>
       <c r="P8" t="str">
         <v>Chưa xuất</v>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -3361,6 +3413,12 @@
       </c>
       <c r="P9" t="str">
         <v>Chưa xuất</v>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -3427,6 +3485,12 @@
       <c r="P10" t="str">
         <v>✅ Đã xuất (kịch bản đầy đủ + ảnh)</v>
       </c>
+      <c r="Q10" t="str">
+        <v>2026-09-10</v>
+      </c>
+      <c r="R10" t="str">
+        <v>2026-09-11</v>
+      </c>
     </row>
     <row r="11" xml:space="preserve">
       <c r="A11">
@@ -3490,10 +3554,16 @@
       <c r="P11" t="str">
         <v>✅ Đã xuất (kịch bản đầy đủ + ảnh)</v>
       </c>
+      <c r="Q11" t="str">
+        <v>2026-09-10</v>
+      </c>
+      <c r="R11" t="str">
+        <v>2026-09-11</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>